<commit_message>
ae agrego lo ultima configuracion de DHCP, y se actualizo la documentacion
</commit_message>
<xml_diff>
--- a/db/ProyectoRedes_Claves.xlsx
+++ b/db/ProyectoRedes_Claves.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perci\Escritorio\8vo_Semestre\Redes\ProyectoFinal\ProyectoRedesFI\db\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel Lara\Music\semestre8\RedesTeoria\Poryecto\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55344C2D-E176-407C-9434-15989513D127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B15D2CCB-EBF6-4330-834B-8C241076A06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{565147E7-335A-4F8E-A460-A735489A30ED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{565147E7-335A-4F8E-A460-A735489A30ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="210">
   <si>
     <t>Contraseñas AP</t>
   </si>
@@ -666,6 +666,9 @@
   </si>
   <si>
     <t>10.0.0.63</t>
+  </si>
+  <si>
+    <t>10.0.0.149</t>
   </si>
 </sst>
 </file>
@@ -739,16 +742,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1086,30 +1089,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C17A4F0-2BEF-4586-A953-5709064D6E13}">
   <dimension ref="B3:N61"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B3" s="4" t="s">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1120,7 +1123,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1131,7 +1134,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
@@ -1142,7 +1145,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
@@ -1153,7 +1156,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>15</v>
       </c>
@@ -1164,7 +1167,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>16</v>
       </c>
@@ -1175,23 +1178,23 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B12" s="4" t="s">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="H12" s="4" t="s">
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="H12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>52</v>
       </c>
@@ -1223,7 +1226,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>51</v>
       </c>
@@ -1255,7 +1258,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>54</v>
       </c>
@@ -1287,7 +1290,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
         <v>55</v>
       </c>
@@ -1319,7 +1322,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>56</v>
       </c>
@@ -1351,7 +1354,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
         <v>57</v>
       </c>
@@ -1368,7 +1371,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B21" s="7" t="s">
         <v>119</v>
       </c>
@@ -1378,593 +1381,597 @@
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B22" s="6" t="s">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B22" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G22" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="I22" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="J22" s="6" t="s">
+      <c r="J22" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="K22" s="6" t="s">
+      <c r="K22" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="L22" s="6" t="s">
+      <c r="L22" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="M22" s="6" t="s">
+      <c r="M22" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="N22" s="6" t="s">
+      <c r="N22" s="5" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B23" s="5" t="s">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="G23" s="5" t="s">
+      <c r="G23" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="L23" s="4">
+        <v>62</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="N23" s="4" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B24" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="L24" s="4">
+        <v>30</v>
+      </c>
+      <c r="M24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="N24" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B25" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="I23" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="J23" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="K23" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="L23" s="5">
-        <v>62</v>
-      </c>
-      <c r="M23" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="N23" s="5" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B24" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="G24" s="5" t="s">
+      <c r="I25" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="L25" s="4">
+        <v>30</v>
+      </c>
+      <c r="M25" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="N25" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B26" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="G26" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="I24" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="J24" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="K24" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="L24" s="5">
-        <v>30</v>
-      </c>
-      <c r="M24" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="N24" s="5" t="s">
+      <c r="I26" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="L26" s="4">
+        <v>14</v>
+      </c>
+      <c r="M26" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="N26" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="L27" s="4">
+        <v>14</v>
+      </c>
+      <c r="M27" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="N27" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B28" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="L28" s="4">
+        <v>2</v>
+      </c>
+      <c r="M28" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="N28" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B29" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="L29" s="4">
+        <v>2</v>
+      </c>
+      <c r="M29" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="N29" s="4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B30" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="L30" s="4">
+        <v>2</v>
+      </c>
+      <c r="M30" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="N30" s="4" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B31" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B32" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B33" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="G33" s="4"/>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B35" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="4"/>
+      <c r="C37" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B38" s="4"/>
+      <c r="C38" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="4"/>
+      <c r="C39" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B40" s="4"/>
+      <c r="C40" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B41" s="4"/>
+      <c r="C41" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B25" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="L25" s="5">
-        <v>30</v>
-      </c>
-      <c r="M25" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="N25" s="5" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B26" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="L26" s="5">
-        <v>14</v>
-      </c>
-      <c r="M26" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="N26" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B27" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="J27" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="K27" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="L27" s="5">
-        <v>14</v>
-      </c>
-      <c r="M27" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="N27" s="5" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B28" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="K28" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="L28" s="5">
-        <v>2</v>
-      </c>
-      <c r="M28" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="N28" s="5" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B29" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="K29" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="L29" s="5">
-        <v>2</v>
-      </c>
-      <c r="M29" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="N29" s="5" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B30" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="I30" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="J30" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="K30" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="L30" s="5">
-        <v>2</v>
-      </c>
-      <c r="M30" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="N30" s="5" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B31" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="G31" s="5"/>
-    </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B32" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="G32" s="5"/>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B33" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="G33" s="5"/>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B34" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B35" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B36" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B37" s="5"/>
-      <c r="C37" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B38" s="5"/>
-      <c r="C38" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B39" s="5"/>
-      <c r="C39" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B40" s="5"/>
-      <c r="C40" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B41" s="5"/>
-      <c r="C41" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="F41" s="5" t="s">
+      <c r="F41" s="4" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B42" s="5"/>
-      <c r="C42" s="5" t="s">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B42" s="4"/>
+      <c r="C42" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C43" s="5" t="s">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C43" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C44" s="5" t="s">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C44" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C45" s="5" t="s">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C45" s="4" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C46" s="5" t="s">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C46" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C47" s="5" t="s">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C47" s="4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C48" s="5" t="s">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C48" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C49" s="5" t="s">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C49" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C50" s="5" t="s">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C50" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C51" s="5" t="s">
+    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C51" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C52" s="5" t="s">
+    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C52" s="4" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C53" s="5" t="s">
+    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C53" s="4" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C54" s="5" t="s">
+    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C54" s="4" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C55" s="5" t="s">
+    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C55" s="4" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C56" s="5" t="s">
+    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C56" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C57" s="5" t="s">
+    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C57" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C58" s="5" t="s">
+    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C58" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C59" s="5" t="s">
+    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C59" s="4" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C60" s="5" t="s">
+    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C60" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C61" s="5"/>
+    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C61" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>